<commit_message>
Update Fall 2026 routine from latest Excel with section revisions
</commit_message>
<xml_diff>
--- a/public/CSE Class Routine Fall-2026.xlsx
+++ b/public/CSE Class Routine Fall-2026.xlsx
@@ -274,16 +274,22 @@
 TH | 803</t>
   </si>
   <si>
-    <t>EEE 2114
-Electronics Devices &amp; Circuits Lab
-1:00-4:00
-IMH | EEE Lab (EEE Dept)</t>
+    <t>EEE 2113
+Electronics Devices &amp; Circuits
+1:00-2:30
+IHS | 1702</t>
   </si>
   <si>
     <t>HUM 3103
 Principles of Management
 09:00 - 12:00
 LM | 1901</t>
+  </si>
+  <si>
+    <t>CSE 3131
+Data Communication &amp; Networking
+3:30-5:00
+TH | 804</t>
   </si>
   <si>
     <t>CSE 3132
@@ -310,22 +316,16 @@
 RBS | 1503</t>
   </si>
   <si>
-    <t>EEE 2113
-Electronics Devices &amp; Circuits
-9:00-10:30
-IMH | 804</t>
-  </si>
-  <si>
     <t>CSE 3219
 Compiler Construction
 10:30 - 12:00
 RBS | 804</t>
   </si>
   <si>
-    <t>CSE 3131
-Data Communication &amp; Networking
-3:30-5:00
-TH | 804</t>
+    <t>EEE 2114
+Electronics Devices &amp; Circuits Lab
+1:00-4:00
+IHS | 903</t>
   </si>
   <si>
     <t>Batch 15, Section B</t>
@@ -424,12 +424,6 @@
 SS | 1702</t>
   </si>
   <si>
-    <t>CSE 1111
-Theory of Computing
-9:00-10:30
-MAR | 1701</t>
-  </si>
-  <si>
     <t>CSE 3151
 Digital Logic Design
 10:30 - 12:00
@@ -446,6 +440,12 @@
 Digital Logic Design Lab
 9:00-12:00
 RBS | 802</t>
+  </si>
+  <si>
+    <t>CSE 1111
+Theory of Computing
+01:30-03:00 |
+MAR | 1401</t>
   </si>
   <si>
     <t>HUM 3103
@@ -562,16 +562,10 @@
 AA | 803</t>
   </si>
   <si>
-    <t>CSE 3108
-Integrated Design Project I
-2:30-4:00
-MAA | Auditorium (13th floor)</t>
-  </si>
-  <si>
     <t>CSE 1111
 Theory of Computing
 9:00-10:30
-MAR | 1704</t>
+MAR | 803</t>
   </si>
   <si>
     <t>CSE 2221
@@ -590,6 +584,11 @@
 Principles of Management
 2:30-4:00
 SS | 1504</t>
+  </si>
+  <si>
+    <t>CSE 3108
+Integrated Design Project I
+MAA | Auditorium (13th floor)</t>
   </si>
   <si>
     <t>MATH 2217
@@ -1146,7 +1145,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1203,8 +1202,18 @@
       <color rgb="FF7F7F7F"/>
       <name val="Times New Roman"/>
     </font>
+    <font>
+      <sz val="10.0"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1279,6 +1288,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFD0E0E3"/>
+        <bgColor rgb="FFD0E0E3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFCFE2F3"/>
         <bgColor rgb="FFCFE2F3"/>
       </patternFill>
@@ -1309,18 +1324,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFCE5CD"/>
+        <bgColor rgb="FFFCE5CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
         <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFCE5CD"/>
-        <bgColor rgb="FFFCE5CD"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="11">
+  <borders count="13">
     <border/>
     <border>
       <left style="thin">
@@ -1407,6 +1422,19 @@
       <left style="thin">
         <color rgb="FF999999"/>
       </left>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
       <right style="thin">
         <color rgb="FF999999"/>
       </right>
@@ -1434,7 +1462,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="62">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1494,28 +1522,57 @@
     <xf borderId="5" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf borderId="1" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="2" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="5" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="1" fillId="12" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="2" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="9" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="11" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="3" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="13" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="14" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="12" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="14" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="15" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="6" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="2" fillId="6" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="13" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="8" fillId="7" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="9" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="3" fillId="12" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="2" fillId="15" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="16" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -1524,22 +1581,28 @@
     <xf borderId="1" fillId="17" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="17" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="18" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="18" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="19" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="18" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="2" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="2" fillId="15" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="16" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="18" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="20" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="2" fillId="18" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="20" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="6" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -1551,29 +1614,29 @@
     <xf borderId="7" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="8" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="2" fillId="19" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="9" fillId="14" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="11" fillId="15" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="10" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="12" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="2" fillId="16" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="17" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="18" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="20" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="18" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="20" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="16" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="17" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1793,10 +1856,10 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="15.0"/>
+    <col customWidth="1" min="2" max="2" width="24.13"/>
     <col customWidth="1" min="3" max="3" width="16.88"/>
     <col customWidth="1" min="4" max="4" width="8.25"/>
-    <col customWidth="1" min="5" max="5" width="16.0"/>
+    <col customWidth="1" min="5" max="5" width="26.25"/>
     <col customWidth="1" min="6" max="6" width="17.88"/>
   </cols>
   <sheetData>
@@ -3009,10 +3072,9 @@
       <c r="D36" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E36" s="18" t="s">
+      <c r="E36" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="F36" s="11"/>
       <c r="G36" s="12"/>
       <c r="H36" s="12"/>
       <c r="I36" s="2"/>
@@ -3038,14 +3100,16 @@
       <c r="A37" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B37" s="21" t="s">
+      <c r="B37" s="22" t="s">
         <v>58</v>
       </c>
       <c r="C37" s="11"/>
       <c r="D37" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E37" s="7"/>
+      <c r="E37" s="23" t="s">
+        <v>59</v>
+      </c>
       <c r="F37" s="7"/>
       <c r="G37" s="12"/>
       <c r="H37" s="12"/>
@@ -3073,18 +3137,18 @@
         <v>14</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C38" s="11"/>
       <c r="D38" s="9" t="s">
         <v>9</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F38" s="7"/>
       <c r="G38" s="12"/>
-      <c r="H38" s="22"/>
+      <c r="H38" s="24"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
@@ -3109,14 +3173,14 @@
         <v>18</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C39" s="11"/>
       <c r="D39" s="9" t="s">
         <v>9</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F39" s="11"/>
       <c r="G39" s="12"/>
@@ -3208,7 +3272,7 @@
       <c r="A42" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B42" s="16" t="s">
+      <c r="B42" s="25" t="s">
         <v>2</v>
       </c>
       <c r="C42" s="16" t="s">
@@ -3249,23 +3313,21 @@
       <c r="Z42" s="2"/>
     </row>
     <row r="43" ht="63.75" customHeight="1">
-      <c r="A43" s="6" t="s">
+      <c r="A43" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="B43" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="C43" s="8" t="s">
+      <c r="B43" s="27"/>
+      <c r="C43" s="28" t="s">
         <v>64</v>
       </c>
       <c r="D43" s="12"/>
       <c r="E43" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F43" s="12"/>
-      <c r="G43" s="23" t="s">
+      <c r="F43" s="29" t="s">
         <v>65</v>
       </c>
+      <c r="G43" s="14"/>
       <c r="H43" s="11"/>
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
@@ -3386,7 +3448,7 @@
       <c r="D47" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E47" s="24" t="s">
+      <c r="E47" s="30" t="s">
         <v>67</v>
       </c>
       <c r="F47" s="11"/>
@@ -3415,7 +3477,7 @@
       <c r="A48" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B48" s="25" t="s">
+      <c r="B48" s="31" t="s">
         <v>68</v>
       </c>
       <c r="C48" s="8" t="s">
@@ -3648,7 +3710,7 @@
         <v>30</v>
       </c>
       <c r="F54" s="12"/>
-      <c r="G54" s="23" t="s">
+      <c r="G54" s="32" t="s">
         <v>79</v>
       </c>
       <c r="H54" s="11"/>
@@ -3834,18 +3896,16 @@
       <c r="A60" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B60" s="8" t="s">
+      <c r="B60" s="8"/>
+      <c r="C60" s="8" t="s">
         <v>83</v>
-      </c>
-      <c r="C60" s="8" t="s">
-        <v>84</v>
       </c>
       <c r="D60" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E60" s="7"/>
+      <c r="E60" s="33"/>
       <c r="F60" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G60" s="12"/>
       <c r="H60" s="12"/>
@@ -3873,13 +3933,15 @@
         <v>18</v>
       </c>
       <c r="B61" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="C61" s="11"/>
+      <c r="D61" s="34" t="s">
+        <v>9</v>
+      </c>
+      <c r="E61" s="35" t="s">
         <v>86</v>
       </c>
-      <c r="C61" s="11"/>
-      <c r="D61" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E61" s="2"/>
       <c r="F61" s="2"/>
       <c r="G61" s="12"/>
       <c r="H61" s="12"/>
@@ -3906,7 +3968,7 @@
       <c r="A62" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B62" s="25" t="s">
+      <c r="B62" s="31" t="s">
         <v>87</v>
       </c>
       <c r="C62" s="8" t="s">
@@ -3915,11 +3977,11 @@
       <c r="D62" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E62" s="10" t="s">
+      <c r="E62" s="36" t="s">
         <v>89</v>
       </c>
-      <c r="F62" s="14"/>
-      <c r="G62" s="26"/>
+      <c r="F62" s="37"/>
+      <c r="G62" s="38"/>
       <c r="H62" s="12"/>
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
@@ -4023,7 +4085,7 @@
       <c r="B65" s="12"/>
       <c r="C65" s="12"/>
       <c r="D65" s="12"/>
-      <c r="E65" s="27" t="s">
+      <c r="E65" s="39" t="s">
         <v>90</v>
       </c>
       <c r="F65" s="11"/>
@@ -4153,7 +4215,7 @@
       <c r="E69" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="F69" s="28" t="s">
+      <c r="F69" s="40" t="s">
         <v>94</v>
       </c>
       <c r="G69" s="12"/>
@@ -4181,10 +4243,10 @@
       <c r="A70" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B70" s="29" t="s">
+      <c r="B70" s="41" t="s">
         <v>95</v>
       </c>
-      <c r="C70" s="30" t="s">
+      <c r="C70" s="42" t="s">
         <v>96</v>
       </c>
       <c r="D70" s="9" t="s">
@@ -4257,16 +4319,16 @@
       <c r="A72" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B72" s="28" t="s">
+      <c r="B72" s="40" t="s">
         <v>101</v>
       </c>
-      <c r="C72" s="28" t="s">
+      <c r="C72" s="40" t="s">
         <v>102</v>
       </c>
       <c r="D72" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E72" s="31" t="s">
+      <c r="E72" s="43" t="s">
         <v>103</v>
       </c>
       <c r="F72" s="11"/>
@@ -4536,7 +4598,7 @@
       <c r="E80" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="F80" s="28" t="s">
+      <c r="F80" s="44" t="s">
         <v>107</v>
       </c>
       <c r="G80" s="12"/>
@@ -4564,20 +4626,18 @@
       <c r="A81" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B81" s="29" t="s">
+      <c r="B81" s="41"/>
+      <c r="C81" s="8" t="s">
         <v>108</v>
-      </c>
-      <c r="C81" s="8" t="s">
-        <v>109</v>
       </c>
       <c r="D81" s="9" t="s">
         <v>9</v>
       </c>
       <c r="E81" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="F81" s="8" t="s">
         <v>110</v>
-      </c>
-      <c r="F81" s="8" t="s">
-        <v>111</v>
       </c>
       <c r="G81" s="12"/>
       <c r="H81" s="12"/>
@@ -4600,11 +4660,13 @@
       <c r="Y81" s="2"/>
       <c r="Z81" s="2"/>
     </row>
-    <row r="82" ht="59.25" customHeight="1">
+    <row r="82" ht="75.75" customHeight="1">
       <c r="A82" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B82" s="12"/>
+      <c r="B82" s="45" t="s">
+        <v>111</v>
+      </c>
       <c r="C82" s="8" t="s">
         <v>112</v>
       </c>
@@ -4791,7 +4853,7 @@
         <v>30</v>
       </c>
       <c r="F87" s="12"/>
-      <c r="G87" s="32"/>
+      <c r="G87" s="46"/>
       <c r="H87" s="11"/>
       <c r="I87" s="2"/>
       <c r="J87" s="2"/>
@@ -4990,7 +5052,7 @@
       <c r="D93" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E93" s="33" t="s">
+      <c r="E93" s="47" t="s">
         <v>123</v>
       </c>
       <c r="F93" s="11"/>
@@ -5324,10 +5386,10 @@
       <c r="A103" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B103" s="34" t="s">
+      <c r="B103" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="C103" s="34" t="s">
+      <c r="C103" s="21" t="s">
         <v>131</v>
       </c>
       <c r="D103" s="9" t="s">
@@ -5373,7 +5435,7 @@
       <c r="D104" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E104" s="33" t="s">
+      <c r="E104" s="47" t="s">
         <v>136</v>
       </c>
       <c r="F104" s="11"/>
@@ -5701,7 +5763,7 @@
       <c r="A114" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B114" s="35"/>
+      <c r="B114" s="48"/>
       <c r="C114" s="7"/>
       <c r="D114" s="9" t="s">
         <v>9</v>
@@ -5773,7 +5835,7 @@
       <c r="A116" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B116" s="36"/>
+      <c r="B116" s="49"/>
       <c r="C116" s="11"/>
       <c r="D116" s="9" t="s">
         <v>9</v>
@@ -5812,7 +5874,7 @@
       <c r="D117" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E117" s="35"/>
+      <c r="E117" s="48"/>
       <c r="F117" s="7"/>
       <c r="G117" s="12"/>
       <c r="H117" s="12"/>
@@ -5924,7 +5986,7 @@
         <v>30</v>
       </c>
       <c r="F120" s="12"/>
-      <c r="G120" s="23" t="s">
+      <c r="G120" s="32" t="s">
         <v>146</v>
       </c>
       <c r="H120" s="11"/>
@@ -6078,7 +6140,7 @@
       <c r="A125" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B125" s="35"/>
+      <c r="B125" s="48"/>
       <c r="C125" s="8" t="s">
         <v>150</v>
       </c>
@@ -6184,7 +6246,7 @@
       <c r="A128" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B128" s="36"/>
+      <c r="B128" s="49"/>
       <c r="C128" s="11"/>
       <c r="D128" s="9" t="s">
         <v>9</v>
@@ -6447,7 +6509,7 @@
       <c r="A136" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B136" s="35"/>
+      <c r="B136" s="48"/>
       <c r="C136" s="8" t="s">
         <v>156</v>
       </c>
@@ -6521,7 +6583,7 @@
       <c r="A138" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B138" s="35"/>
+      <c r="B138" s="48"/>
       <c r="C138" s="8" t="s">
         <v>161</v>
       </c>
@@ -6562,7 +6624,7 @@
       <c r="D139" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E139" s="36"/>
+      <c r="E139" s="49"/>
       <c r="F139" s="11"/>
       <c r="G139" s="12"/>
       <c r="H139" s="12"/>
@@ -6820,7 +6882,7 @@
       <c r="A147" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B147" s="36"/>
+      <c r="B147" s="49"/>
       <c r="C147" s="11"/>
       <c r="D147" s="9" t="s">
         <v>9</v>
@@ -6856,7 +6918,7 @@
       <c r="A148" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B148" s="35"/>
+      <c r="B148" s="48"/>
       <c r="C148" s="8" t="s">
         <v>161</v>
       </c>
@@ -6928,7 +6990,7 @@
       <c r="A150" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B150" s="35"/>
+      <c r="B150" s="48"/>
       <c r="C150" s="7"/>
       <c r="D150" s="9" t="s">
         <v>9</v>
@@ -7197,7 +7259,7 @@
       <c r="A158" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B158" s="27" t="s">
+      <c r="B158" s="39" t="s">
         <v>172</v>
       </c>
       <c r="C158" s="11"/>
@@ -7263,7 +7325,7 @@
       <c r="A160" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B160" s="23" t="s">
+      <c r="B160" s="32" t="s">
         <v>173</v>
       </c>
       <c r="C160" s="11"/>
@@ -7412,7 +7474,7 @@
       <c r="B164" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C164" s="28" t="s">
+      <c r="C164" s="40" t="s">
         <v>177</v>
       </c>
       <c r="D164" s="12"/>
@@ -7512,7 +7574,7 @@
         <v>6</v>
       </c>
       <c r="G167" s="5"/>
-      <c r="H167" s="37"/>
+      <c r="H167" s="50"/>
       <c r="I167" s="2"/>
       <c r="J167" s="2"/>
       <c r="K167" s="2"/>
@@ -7541,8 +7603,8 @@
       <c r="D168" s="2"/>
       <c r="E168" s="12"/>
       <c r="F168" s="2"/>
-      <c r="G168" s="38"/>
-      <c r="H168" s="39"/>
+      <c r="G168" s="51"/>
+      <c r="H168" s="52"/>
       <c r="I168" s="2"/>
       <c r="J168" s="2"/>
       <c r="K168" s="2"/>
@@ -7566,7 +7628,7 @@
       <c r="A169" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B169" s="23" t="s">
+      <c r="B169" s="32" t="s">
         <v>179</v>
       </c>
       <c r="C169" s="11"/>
@@ -7578,7 +7640,7 @@
         <v>180</v>
       </c>
       <c r="G169" s="12"/>
-      <c r="H169" s="40"/>
+      <c r="H169" s="53"/>
       <c r="I169" s="2"/>
       <c r="J169" s="2"/>
       <c r="K169" s="2"/>
@@ -7617,7 +7679,6 @@
       <c r="F170" s="11"/>
       <c r="G170" s="12"/>
       <c r="H170" s="12"/>
-      <c r="I170" s="2"/>
       <c r="J170" s="2"/>
       <c r="K170" s="2"/>
       <c r="L170" s="2"/>
@@ -7640,7 +7701,7 @@
       <c r="A171" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B171" s="41" t="s">
+      <c r="B171" s="54" t="s">
         <v>172</v>
       </c>
       <c r="C171" s="11"/>
@@ -7651,7 +7712,6 @@
       <c r="F171" s="7"/>
       <c r="G171" s="12"/>
       <c r="H171" s="12"/>
-      <c r="I171" s="2"/>
       <c r="J171" s="2"/>
       <c r="K171" s="2"/>
       <c r="L171" s="2"/>
@@ -7788,11 +7848,11 @@
       <c r="E175" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F175" s="42" t="s">
+      <c r="F175" s="55" t="s">
         <v>184</v>
       </c>
-      <c r="G175" s="43"/>
-      <c r="H175" s="44"/>
+      <c r="G175" s="56"/>
+      <c r="H175" s="57"/>
       <c r="I175" s="2"/>
       <c r="J175" s="2"/>
       <c r="K175" s="2"/>
@@ -7944,7 +8004,7 @@
       <c r="D180" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E180" s="45" t="s">
+      <c r="E180" s="58" t="s">
         <v>186</v>
       </c>
       <c r="F180" s="11"/>
@@ -7982,7 +8042,7 @@
       <c r="D181" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E181" s="23" t="s">
+      <c r="E181" s="32" t="s">
         <v>189</v>
       </c>
       <c r="F181" s="11"/>
@@ -8159,7 +8219,7 @@
       <c r="E186" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F186" s="23" t="s">
+      <c r="F186" s="32" t="s">
         <v>191</v>
       </c>
       <c r="G186" s="14"/>
@@ -8278,7 +8338,7 @@
       <c r="A190" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B190" s="45" t="s">
+      <c r="B190" s="58" t="s">
         <v>193</v>
       </c>
       <c r="C190" s="11"/>
@@ -8288,7 +8348,7 @@
       <c r="E190" s="8" t="s">
         <v>194</v>
       </c>
-      <c r="F190" s="46" t="s">
+      <c r="F190" s="59" t="s">
         <v>195</v>
       </c>
       <c r="G190" s="12"/>
@@ -8325,7 +8385,7 @@
       <c r="D191" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E191" s="47" t="s">
+      <c r="E191" s="60" t="s">
         <v>198</v>
       </c>
       <c r="F191" s="11"/>
@@ -8363,7 +8423,7 @@
       <c r="D192" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E192" s="46" t="s">
+      <c r="E192" s="59" t="s">
         <v>200</v>
       </c>
       <c r="F192" s="2"/>
@@ -8687,7 +8747,7 @@
       <c r="A202" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B202" s="46" t="s">
+      <c r="B202" s="59" t="s">
         <v>202</v>
       </c>
       <c r="C202" s="8" t="s">
@@ -8727,14 +8787,14 @@
       <c r="A203" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B203" s="46" t="s">
+      <c r="B203" s="59" t="s">
         <v>202</v>
       </c>
       <c r="C203" s="7"/>
       <c r="D203" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E203" s="47" t="s">
+      <c r="E203" s="60" t="s">
         <v>198</v>
       </c>
       <c r="F203" s="11"/>
@@ -8772,7 +8832,7 @@
       <c r="D204" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E204" s="48"/>
+      <c r="E204" s="61"/>
       <c r="F204" s="11"/>
       <c r="G204" s="12"/>
       <c r="H204" s="12"/>
@@ -31116,114 +31176,113 @@
       <c r="Z1000" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="107">
+  <mergeCells count="106">
+    <mergeCell ref="B73:H73"/>
+    <mergeCell ref="B74:H74"/>
+    <mergeCell ref="A78:H78"/>
+    <mergeCell ref="B80:C80"/>
+    <mergeCell ref="B85:H85"/>
+    <mergeCell ref="G87:H87"/>
+    <mergeCell ref="A89:H89"/>
+    <mergeCell ref="B87:C87"/>
+    <mergeCell ref="B91:C91"/>
+    <mergeCell ref="E92:F92"/>
+    <mergeCell ref="E93:F93"/>
+    <mergeCell ref="B95:H95"/>
+    <mergeCell ref="B96:H96"/>
+    <mergeCell ref="A100:H100"/>
+    <mergeCell ref="B116:C116"/>
+    <mergeCell ref="B120:C120"/>
+    <mergeCell ref="E102:F102"/>
+    <mergeCell ref="E104:F104"/>
+    <mergeCell ref="B106:C106"/>
+    <mergeCell ref="B107:H107"/>
+    <mergeCell ref="A111:H111"/>
+    <mergeCell ref="E116:F116"/>
+    <mergeCell ref="B118:H118"/>
+    <mergeCell ref="E136:F136"/>
+    <mergeCell ref="B137:C137"/>
+    <mergeCell ref="E139:F139"/>
+    <mergeCell ref="B140:H140"/>
+    <mergeCell ref="A144:H144"/>
+    <mergeCell ref="B147:C147"/>
+    <mergeCell ref="B149:C149"/>
+    <mergeCell ref="E150:F150"/>
+    <mergeCell ref="B151:H151"/>
+    <mergeCell ref="A155:H155"/>
+    <mergeCell ref="E157:F157"/>
+    <mergeCell ref="B158:C158"/>
+    <mergeCell ref="B160:C160"/>
+    <mergeCell ref="B161:H161"/>
+    <mergeCell ref="B162:H162"/>
+    <mergeCell ref="A166:H166"/>
+    <mergeCell ref="B169:C169"/>
+    <mergeCell ref="E170:F170"/>
+    <mergeCell ref="B171:C171"/>
+    <mergeCell ref="B172:H172"/>
+    <mergeCell ref="B173:H173"/>
+    <mergeCell ref="F175:G175"/>
+    <mergeCell ref="A177:H177"/>
+    <mergeCell ref="E180:F180"/>
+    <mergeCell ref="E181:F181"/>
+    <mergeCell ref="E182:F182"/>
+    <mergeCell ref="B183:H183"/>
+    <mergeCell ref="B184:H184"/>
+    <mergeCell ref="E203:F203"/>
+    <mergeCell ref="E204:F204"/>
+    <mergeCell ref="B205:H205"/>
+    <mergeCell ref="B206:H206"/>
+    <mergeCell ref="F186:H186"/>
+    <mergeCell ref="A188:H188"/>
+    <mergeCell ref="B190:C190"/>
+    <mergeCell ref="E191:F191"/>
+    <mergeCell ref="B194:H194"/>
+    <mergeCell ref="B195:H195"/>
+    <mergeCell ref="A199:H199"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="B8:H8"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:H19"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="B30:H30"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="E39:F39"/>
     <mergeCell ref="B40:H40"/>
     <mergeCell ref="B41:H41"/>
-    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="F43:H43"/>
+    <mergeCell ref="A45:H45"/>
     <mergeCell ref="E47:F47"/>
     <mergeCell ref="E49:F49"/>
-    <mergeCell ref="A45:H45"/>
     <mergeCell ref="B50:C50"/>
     <mergeCell ref="B52:H52"/>
     <mergeCell ref="B54:C54"/>
+    <mergeCell ref="E65:F65"/>
+    <mergeCell ref="E72:F72"/>
     <mergeCell ref="G54:H54"/>
+    <mergeCell ref="A56:H56"/>
+    <mergeCell ref="B61:C61"/>
     <mergeCell ref="E62:F62"/>
     <mergeCell ref="B63:H63"/>
-    <mergeCell ref="A56:H56"/>
-    <mergeCell ref="B118:H118"/>
+    <mergeCell ref="A67:H67"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="G120:H120"/>
     <mergeCell ref="A122:H122"/>
-    <mergeCell ref="E102:F102"/>
-    <mergeCell ref="E104:F104"/>
-    <mergeCell ref="B106:C106"/>
-    <mergeCell ref="B107:H107"/>
-    <mergeCell ref="B116:C116"/>
-    <mergeCell ref="E116:F116"/>
-    <mergeCell ref="A111:H111"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="B30:H30"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="A34:H34"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="E72:F72"/>
-    <mergeCell ref="B73:H73"/>
-    <mergeCell ref="B74:H74"/>
-    <mergeCell ref="B80:C80"/>
-    <mergeCell ref="B85:H85"/>
-    <mergeCell ref="A78:H78"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B7:H7"/>
-    <mergeCell ref="B8:H8"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:H19"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="E65:F65"/>
-    <mergeCell ref="A67:H67"/>
-    <mergeCell ref="B96:H96"/>
-    <mergeCell ref="A100:H100"/>
-    <mergeCell ref="B87:C87"/>
-    <mergeCell ref="G87:H87"/>
-    <mergeCell ref="B91:C91"/>
-    <mergeCell ref="E92:F92"/>
-    <mergeCell ref="E93:F93"/>
-    <mergeCell ref="B95:H95"/>
-    <mergeCell ref="A89:H89"/>
-    <mergeCell ref="E182:F182"/>
-    <mergeCell ref="E203:F203"/>
-    <mergeCell ref="E204:F204"/>
-    <mergeCell ref="B184:H184"/>
-    <mergeCell ref="B190:C190"/>
-    <mergeCell ref="E191:F191"/>
-    <mergeCell ref="B194:H194"/>
-    <mergeCell ref="B195:H195"/>
-    <mergeCell ref="B205:H205"/>
-    <mergeCell ref="B206:H206"/>
-    <mergeCell ref="A199:H199"/>
-    <mergeCell ref="B137:C137"/>
-    <mergeCell ref="B147:C147"/>
-    <mergeCell ref="B149:C149"/>
-    <mergeCell ref="B158:C158"/>
-    <mergeCell ref="B160:C160"/>
-    <mergeCell ref="B169:C169"/>
-    <mergeCell ref="B171:C171"/>
-    <mergeCell ref="E136:F136"/>
-    <mergeCell ref="E139:F139"/>
-    <mergeCell ref="E150:F150"/>
-    <mergeCell ref="E157:F157"/>
-    <mergeCell ref="E170:F170"/>
-    <mergeCell ref="E180:F180"/>
-    <mergeCell ref="E181:F181"/>
-    <mergeCell ref="B140:H140"/>
-    <mergeCell ref="A144:H144"/>
-    <mergeCell ref="B120:C120"/>
-    <mergeCell ref="G120:H120"/>
     <mergeCell ref="B124:C124"/>
     <mergeCell ref="E124:F124"/>
     <mergeCell ref="B128:C128"/>
     <mergeCell ref="B129:H129"/>
     <mergeCell ref="A133:H133"/>
-    <mergeCell ref="B162:H162"/>
-    <mergeCell ref="A166:H166"/>
-    <mergeCell ref="B151:H151"/>
-    <mergeCell ref="B161:H161"/>
-    <mergeCell ref="B172:H172"/>
-    <mergeCell ref="B173:H173"/>
-    <mergeCell ref="F175:G175"/>
-    <mergeCell ref="B183:H183"/>
-    <mergeCell ref="A155:H155"/>
-    <mergeCell ref="A177:H177"/>
-    <mergeCell ref="F186:H186"/>
-    <mergeCell ref="A188:H188"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>